<commit_message>
Updated after changing account name pulling
</commit_message>
<xml_diff>
--- a/data/info_for_pdf.xlsx
+++ b/data/info_for_pdf.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/michaelmolenaar/Desktop/BROGAARD/Gaard/Gaard Reporting System/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6BF861B-7D05-714F-8514-17E2571A53AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECCEEB53-3A64-384F-B74D-D11A51EAA272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="41120" windowHeight="25800" xr2:uid="{6D522E3E-A00D-E248-87E0-EF62B3A29ADA}"/>
   </bookViews>

</xml_diff>